<commit_message>
them toi bai 6
</commit_message>
<xml_diff>
--- a/Lab2/PhanVungTuongDuong.xlsx
+++ b/Lab2/PhanVungTuongDuong.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="18350" windowHeight="6080" activeTab="6"/>
+    <workbookView windowWidth="18350" windowHeight="6800" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="Bai1" sheetId="1" r:id="rId1"/>
@@ -13,7 +13,7 @@
     <sheet name="Bai4" sheetId="4" r:id="rId4"/>
     <sheet name="Bai5" sheetId="5" r:id="rId5"/>
     <sheet name="Bai6" sheetId="6" r:id="rId6"/>
-    <sheet name="Sheet7" sheetId="7" r:id="rId7"/>
+    <sheet name="Bai7" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="468" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="449" uniqueCount="187">
   <si>
     <t>TEST CASE ID:</t>
   </si>
@@ -503,130 +503,91 @@
     <t>Validate student score analysis file</t>
   </si>
   <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>Gender</t>
-  </si>
-  <si>
-    <t>Scores (5 subjects)</t>
+    <t>Test Data Description</t>
   </si>
   <si>
     <t>File input được tải lên hệ thống</t>
   </si>
   <si>
-    <t>An</t>
-  </si>
-  <si>
-    <t>M</t>
-  </si>
-  <si>
-    <t>6,7,8,5,6</t>
-  </si>
-  <si>
-    <t>Lên lớp</t>
+    <t>File hợp lệ (≤100 dòng)</t>
   </si>
   <si>
     <t>File có định dạng đúng</t>
   </si>
   <si>
-    <t>Bình</t>
-  </si>
-  <si>
-    <t>F</t>
-  </si>
-  <si>
-    <t>4,5,3,6,4</t>
+    <t>File có tên sinh viên &gt;20 ký tự</t>
+  </si>
+  <si>
+    <t>Chương trình phân tích sẵn sàng</t>
+  </si>
+  <si>
+    <t>File có giới tính không hợp lệ</t>
+  </si>
+  <si>
+    <t>File có điểm &lt;0</t>
+  </si>
+  <si>
+    <t>File có điểm &gt;10</t>
+  </si>
+  <si>
+    <t>File có điểm trung bình &lt;5</t>
+  </si>
+  <si>
+    <t>File có điểm trung bình ≥5</t>
+  </si>
+  <si>
+    <t>Tên ≤ 20 ký tự</t>
+  </si>
+  <si>
+    <t>Giới tính: M / F</t>
+  </si>
+  <si>
+    <t>Điểm từng môn: 0 – 10</t>
+  </si>
+  <si>
+    <t>Số dòng ≤ 100</t>
+  </si>
+  <si>
+    <t>Tên &gt; 20 ký tự</t>
+  </si>
+  <si>
+    <t>Giới tính khác M/F</t>
+  </si>
+  <si>
+    <t>Điểm &lt;0 hoặc &gt;10</t>
+  </si>
+  <si>
+    <t>Input Data</t>
+  </si>
+  <si>
+    <t>File hợp lệ</t>
+  </si>
+  <si>
+    <t>An – M – 6,7,8,5,6</t>
+  </si>
+  <si>
+    <t>Tính điểm TB</t>
+  </si>
+  <si>
+    <t>Điểm TB &lt;5</t>
+  </si>
+  <si>
+    <t>Bình – F – 4,5,3,6,4</t>
   </si>
   <si>
     <t>Không lên lớp</t>
   </si>
   <si>
-    <t>Chương trình phân tích sẵn sàng</t>
-  </si>
-  <si>
-    <t>LongLongLongLongLong1</t>
-  </si>
-  <si>
-    <t>8,8,8,8,8</t>
-  </si>
-  <si>
-    <t>Lỗi tên</t>
-  </si>
-  <si>
-    <t>Dũng</t>
+    <t>Tên quá dài</t>
+  </si>
+  <si>
+    <t>Long…</t>
+  </si>
+  <si>
+    <t>Sai giới tính</t>
   </si>
   <si>
     <t>X</t>
-  </si>
-  <si>
-    <t>7,7,7,7,7</t>
-  </si>
-  <si>
-    <t>Lỗi giới tính</t>
-  </si>
-  <si>
-    <t>Hà</t>
-  </si>
-  <si>
-    <t>11,9,8,7,6</t>
-  </si>
-  <si>
-    <t>Lỗi điểm</t>
-  </si>
-  <si>
-    <t>Mai</t>
-  </si>
-  <si>
-    <t>-1,6,7,8,9</t>
-  </si>
-  <si>
-    <t>Tên ≤ 20 ký tự</t>
-  </si>
-  <si>
-    <t>Giới tính: M / F</t>
-  </si>
-  <si>
-    <t>Điểm từng môn: 0 – 10</t>
-  </si>
-  <si>
-    <t>Số dòng ≤ 100</t>
-  </si>
-  <si>
-    <t>Tên &gt; 20 ký tự</t>
-  </si>
-  <si>
-    <t>Giới tính khác M/F</t>
-  </si>
-  <si>
-    <t>Điểm &lt;0 hoặc &gt;10</t>
-  </si>
-  <si>
-    <t>Input Data</t>
-  </si>
-  <si>
-    <t>File hợp lệ</t>
-  </si>
-  <si>
-    <t>An – M – 6,7,8,5,6</t>
-  </si>
-  <si>
-    <t>Tính điểm TB</t>
-  </si>
-  <si>
-    <t>Điểm TB &lt;5</t>
-  </si>
-  <si>
-    <t>Bình – F – 4,5,3,6,4</t>
-  </si>
-  <si>
-    <t>Tên quá dài</t>
-  </si>
-  <si>
-    <t>Long…</t>
-  </si>
-  <si>
-    <t>Sai giới tính</t>
   </si>
   <si>
     <t>Điểm &gt;10</t>
@@ -1262,7 +1223,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1275,27 +1236,30 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="58" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1309,18 +1273,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1875,7 +1830,7 @@
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
       <c r="E1" s="3" t="s">
@@ -1889,13 +1844,13 @@
       <c r="B2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="2" t="s">
         <v>7</v>
       </c>
       <c r="G2" s="3" t="s">
@@ -1912,10 +1867,10 @@
       <c r="C4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="4">
         <v>46028</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="2" t="s">
         <v>11</v>
       </c>
       <c r="F4" s="3" t="s">
@@ -1923,90 +1878,90 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="17" t="s">
+      <c r="A6" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="17" t="s">
+      <c r="B6" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="17" t="s">
+      <c r="D6" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="17" t="s">
+      <c r="E6" s="5" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="7" ht="29" spans="1:5">
-      <c r="A7" s="18">
+      <c r="A7" s="17">
         <v>1</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="B7" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="18">
+      <c r="D7" s="17">
         <v>1</v>
       </c>
-      <c r="E7" s="18" t="s">
+      <c r="E7" s="17" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="18">
+      <c r="A8" s="17">
         <v>2</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="B8" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="18">
+      <c r="D8" s="17">
         <v>2</v>
       </c>
-      <c r="E8" s="18" t="s">
+      <c r="E8" s="17" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="9" ht="29" spans="1:5">
-      <c r="A9" s="18">
+      <c r="A9" s="17">
         <v>3</v>
       </c>
-      <c r="B9" s="18" t="s">
+      <c r="B9" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="D9" s="18">
+      <c r="D9" s="17">
         <v>3</v>
       </c>
-      <c r="E9" s="18" t="s">
+      <c r="E9" s="17" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="10" spans="4:5">
-      <c r="D10" s="18">
+      <c r="D10" s="17">
         <v>4</v>
       </c>
-      <c r="E10" s="18" t="s">
+      <c r="E10" s="17" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="11" spans="4:5">
-      <c r="D11" s="18">
+      <c r="D11" s="17">
         <v>5</v>
       </c>
-      <c r="E11" s="18" t="s">
+      <c r="E11" s="17" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="12" spans="4:5">
-      <c r="D12" s="18">
+      <c r="D12" s="17">
         <v>6</v>
       </c>
-      <c r="E12" s="18" t="s">
+      <c r="E12" s="17" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="13" spans="4:5">
-      <c r="D13" s="18">
+      <c r="D13" s="17">
         <v>7</v>
       </c>
-      <c r="E13" s="18" t="s">
+      <c r="E13" s="17" t="s">
         <v>25</v>
       </c>
     </row>
@@ -2066,132 +2021,132 @@
       </c>
     </row>
     <row r="23" spans="1:6">
-      <c r="A23" s="19" t="s">
+      <c r="A23" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="B23" s="19" t="s">
+      <c r="B23" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="C23" s="19" t="s">
+      <c r="C23" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="D23" s="19" t="s">
+      <c r="D23" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="E23" s="19"/>
-      <c r="F23" s="19"/>
+      <c r="E23" s="10"/>
+      <c r="F23" s="10"/>
     </row>
     <row r="24" ht="29" spans="1:6">
-      <c r="A24" s="18" t="s">
+      <c r="A24" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="B24" s="18" t="s">
+      <c r="B24" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="C24" s="18" t="s">
+      <c r="C24" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="D24" s="18" t="s">
+      <c r="D24" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="E24" s="18"/>
-      <c r="F24" s="18"/>
+      <c r="E24" s="17"/>
+      <c r="F24" s="17"/>
     </row>
     <row r="25" spans="1:6">
-      <c r="A25" s="18" t="s">
+      <c r="A25" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="B25" s="18" t="s">
+      <c r="B25" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="C25" s="18" t="s">
+      <c r="C25" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="D25" s="18" t="s">
+      <c r="D25" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="E25" s="18"/>
-      <c r="F25" s="18"/>
+      <c r="E25" s="17"/>
+      <c r="F25" s="17"/>
     </row>
     <row r="26" spans="1:6">
-      <c r="A26" s="18" t="s">
+      <c r="A26" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="B26" s="18" t="s">
+      <c r="B26" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="C26" s="18" t="s">
+      <c r="C26" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="D26" s="18" t="s">
+      <c r="D26" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="E26" s="18"/>
-      <c r="F26" s="18"/>
+      <c r="E26" s="17"/>
+      <c r="F26" s="17"/>
     </row>
     <row r="27" spans="1:6">
-      <c r="A27" s="18" t="s">
+      <c r="A27" s="17" t="s">
         <v>47</v>
       </c>
-      <c r="B27" s="18" t="s">
+      <c r="B27" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="C27" s="18" t="s">
+      <c r="C27" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="D27" s="18" t="s">
+      <c r="D27" s="17" t="s">
         <v>49</v>
       </c>
-      <c r="E27" s="18"/>
-      <c r="F27" s="18"/>
+      <c r="E27" s="17"/>
+      <c r="F27" s="17"/>
     </row>
     <row r="28" spans="1:6">
-      <c r="A28" s="18" t="s">
+      <c r="A28" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="B28" s="18" t="s">
+      <c r="B28" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="C28" s="18" t="s">
+      <c r="C28" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="D28" s="18" t="s">
+      <c r="D28" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="E28" s="18"/>
-      <c r="F28" s="18"/>
+      <c r="E28" s="17"/>
+      <c r="F28" s="17"/>
     </row>
     <row r="29" spans="1:6">
-      <c r="A29" s="18" t="s">
+      <c r="A29" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="B29" s="18" t="s">
+      <c r="B29" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="C29" s="18" t="s">
+      <c r="C29" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="D29" s="18" t="s">
+      <c r="D29" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="E29" s="18"/>
-      <c r="F29" s="18"/>
+      <c r="E29" s="17"/>
+      <c r="F29" s="17"/>
     </row>
     <row r="30" ht="29" spans="1:6">
-      <c r="A30" s="18" t="s">
+      <c r="A30" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="B30" s="18" t="s">
+      <c r="B30" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="C30" s="18" t="s">
+      <c r="C30" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="D30" s="18" t="s">
+      <c r="D30" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="E30" s="18"/>
-      <c r="F30" s="18"/>
+      <c r="E30" s="17"/>
+      <c r="F30" s="17"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2235,7 +2190,7 @@
       <c r="B2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D2" s="3" t="s">
@@ -2258,10 +2213,10 @@
       <c r="C4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="4">
         <v>46028</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="2" t="s">
         <v>11</v>
       </c>
       <c r="F4" s="3" t="s">
@@ -2269,68 +2224,68 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="5" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="7">
+      <c r="A7" s="8">
         <v>1</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="D7" s="7">
+      <c r="D7" s="8">
         <v>1</v>
       </c>
-      <c r="E7" s="7">
+      <c r="E7" s="8">
         <v>123456</v>
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="7">
+      <c r="A8" s="8">
         <v>2</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="D8" s="7">
+      <c r="D8" s="8">
         <v>2</v>
       </c>
-      <c r="E8" s="7">
+      <c r="E8" s="8">
         <v>1234567890</v>
       </c>
     </row>
     <row r="9" spans="4:5">
-      <c r="D9" s="7">
+      <c r="D9" s="8">
         <v>3</v>
       </c>
-      <c r="E9" s="7">
+      <c r="E9" s="8">
         <v>12345</v>
       </c>
     </row>
     <row r="10" spans="4:5">
-      <c r="D10" s="7">
+      <c r="D10" s="8">
         <v>4</v>
       </c>
-      <c r="E10" s="7">
+      <c r="E10" s="8">
         <v>12345678901</v>
       </c>
     </row>
     <row r="11" spans="4:5">
-      <c r="D11" s="7">
+      <c r="D11" s="8">
         <v>5</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="E11" s="8" t="s">
         <v>62</v>
       </c>
     </row>
@@ -2382,100 +2337,100 @@
       </c>
     </row>
     <row r="20" spans="1:6">
-      <c r="A20" s="8" t="s">
+      <c r="A20" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="B20" s="8" t="s">
+      <c r="B20" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="C20" s="8" t="s">
+      <c r="C20" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="D20" s="8" t="s">
+      <c r="D20" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="E20" s="8"/>
-      <c r="F20" s="8"/>
+      <c r="E20" s="10"/>
+      <c r="F20" s="10"/>
     </row>
     <row r="21" spans="1:6">
-      <c r="A21" s="7" t="s">
+      <c r="A21" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="B21" s="7" t="s">
+      <c r="B21" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="C21" s="7">
+      <c r="C21" s="8">
         <v>123456</v>
       </c>
-      <c r="D21" s="7" t="s">
+      <c r="D21" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="E21" s="7"/>
-      <c r="F21" s="7"/>
+      <c r="E21" s="8"/>
+      <c r="F21" s="8"/>
     </row>
     <row r="22" spans="1:6">
-      <c r="A22" s="7" t="s">
+      <c r="A22" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="B22" s="7" t="s">
+      <c r="B22" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="C22" s="7">
+      <c r="C22" s="8">
         <v>1234567890</v>
       </c>
-      <c r="D22" s="7" t="s">
+      <c r="D22" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="E22" s="7"/>
-      <c r="F22" s="7"/>
+      <c r="E22" s="8"/>
+      <c r="F22" s="8"/>
     </row>
     <row r="23" spans="1:6">
-      <c r="A23" s="7" t="s">
+      <c r="A23" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="B23" s="7" t="s">
+      <c r="B23" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="C23" s="7">
+      <c r="C23" s="8">
         <v>12345</v>
       </c>
-      <c r="D23" s="7" t="s">
+      <c r="D23" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="E23" s="7"/>
-      <c r="F23" s="7"/>
+      <c r="E23" s="8"/>
+      <c r="F23" s="8"/>
     </row>
     <row r="24" spans="1:6">
-      <c r="A24" s="7" t="s">
+      <c r="A24" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="B24" s="7" t="s">
+      <c r="B24" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="C24" s="7">
+      <c r="C24" s="8">
         <v>12345678901</v>
       </c>
-      <c r="D24" s="7" t="s">
+      <c r="D24" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="E24" s="7"/>
-      <c r="F24" s="7"/>
+      <c r="E24" s="8"/>
+      <c r="F24" s="8"/>
     </row>
     <row r="25" spans="1:6">
-      <c r="A25" s="7" t="s">
+      <c r="A25" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="B25" s="7" t="s">
+      <c r="B25" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="C25" s="7" t="s">
+      <c r="C25" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="D25" s="7" t="s">
+      <c r="D25" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="E25" s="7"/>
-      <c r="F25" s="7"/>
+      <c r="E25" s="8"/>
+      <c r="F25" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2520,7 +2475,7 @@
       <c r="B2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D2" s="3" t="s">
@@ -2551,10 +2506,10 @@
       <c r="C4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="4">
         <v>46028</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="2" t="s">
         <v>11</v>
       </c>
       <c r="F4" s="3" t="s">
@@ -2562,73 +2517,73 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="10" t="s">
+      <c r="E6" s="5" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="11">
+      <c r="A7" s="12">
         <v>1</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="12" t="s">
         <v>79</v>
       </c>
-      <c r="D7" s="11">
+      <c r="D7" s="12">
         <v>1</v>
       </c>
-      <c r="E7" s="12">
+      <c r="E7" s="13">
         <v>0.333333333333333</v>
       </c>
     </row>
     <row r="8" ht="29" spans="1:5">
-      <c r="A8" s="11">
+      <c r="A8" s="12">
         <v>2</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="12" t="s">
         <v>80</v>
       </c>
-      <c r="D8" s="11">
+      <c r="D8" s="12">
         <v>2</v>
       </c>
-      <c r="E8" s="12">
+      <c r="E8" s="13">
         <v>0.395833333333333</v>
       </c>
     </row>
     <row r="9" spans="4:5">
-      <c r="D9" s="11">
+      <c r="D9" s="12">
         <v>3</v>
       </c>
-      <c r="E9" s="12">
+      <c r="E9" s="13">
         <v>0.666666666666667</v>
       </c>
     </row>
     <row r="10" spans="4:5">
-      <c r="D10" s="11">
+      <c r="D10" s="12">
         <v>4</v>
       </c>
-      <c r="E10" s="12">
+      <c r="E10" s="13">
         <v>0.813194444444444</v>
       </c>
     </row>
     <row r="11" spans="4:5">
-      <c r="D11" s="11">
+      <c r="D11" s="12">
         <v>5</v>
       </c>
-      <c r="E11" s="13">
+      <c r="E11" s="14">
         <v>1.04166666666667</v>
       </c>
     </row>
     <row r="12" spans="1:1">
-      <c r="A12" s="14" t="s">
+      <c r="A12" s="15" t="s">
         <v>63</v>
       </c>
     </row>
@@ -2667,82 +2622,82 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="15" t="s">
+      <c r="A19" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="B19" s="15" t="s">
+      <c r="B19" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="C19" s="15" t="s">
+      <c r="C19" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="D19" s="15"/>
-      <c r="E19" s="15"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="10"/>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="11" t="s">
+      <c r="A20" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="B20" s="12">
+      <c r="B20" s="13">
         <v>0.333333333333333</v>
       </c>
-      <c r="C20" s="11" t="s">
+      <c r="C20" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="D20" s="11"/>
-      <c r="E20" s="11"/>
+      <c r="D20" s="12"/>
+      <c r="E20" s="12"/>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="11" t="s">
+      <c r="A21" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="B21" s="12">
+      <c r="B21" s="13">
         <v>0.395833333333333</v>
       </c>
-      <c r="C21" s="11" t="s">
+      <c r="C21" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="D21" s="11"/>
-      <c r="E21" s="11"/>
+      <c r="D21" s="12"/>
+      <c r="E21" s="12"/>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="11" t="s">
+      <c r="A22" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="B22" s="12">
+      <c r="B22" s="13">
         <v>0.666666666666667</v>
       </c>
-      <c r="C22" s="11" t="s">
+      <c r="C22" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="D22" s="11"/>
-      <c r="E22" s="11"/>
+      <c r="D22" s="12"/>
+      <c r="E22" s="12"/>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="11" t="s">
+      <c r="A23" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="B23" s="12">
+      <c r="B23" s="13">
         <v>0.813194444444444</v>
       </c>
-      <c r="C23" s="11" t="s">
+      <c r="C23" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="D23" s="11"/>
-      <c r="E23" s="11"/>
+      <c r="D23" s="12"/>
+      <c r="E23" s="12"/>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="11" t="s">
+      <c r="A24" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="B24" s="13">
+      <c r="B24" s="14">
         <v>1.04166666666667</v>
       </c>
-      <c r="C24" s="11" t="s">
+      <c r="C24" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="D24" s="11"/>
-      <c r="E24" s="11"/>
+      <c r="D24" s="12"/>
+      <c r="E24" s="12"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2786,7 +2741,7 @@
       <c r="B2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D2" s="3" t="s">
@@ -2809,10 +2764,10 @@
       <c r="C4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="4">
         <v>46028</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="2" t="s">
         <v>11</v>
       </c>
       <c r="F4" s="3" t="s">
@@ -2820,58 +2775,58 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="7" ht="29" spans="1:5">
-      <c r="A7" s="7">
+      <c r="A7" s="8">
         <v>1</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="D7" s="7">
+      <c r="D7" s="8">
         <v>1</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="8" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="8" ht="43.5" spans="1:5">
-      <c r="A8" s="7">
+      <c r="A8" s="8">
         <v>2</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="D8" s="7">
+      <c r="D8" s="8">
         <v>2</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="8" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="9" ht="29" spans="1:5">
-      <c r="A9" s="7">
+      <c r="A9" s="8">
         <v>3</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="D9" s="7">
+      <c r="D9" s="8">
         <v>3</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="8" t="s">
         <v>91</v>
       </c>
     </row>
@@ -2947,148 +2902,148 @@
       </c>
     </row>
     <row r="22" spans="1:6">
-      <c r="A22" s="8" t="s">
+      <c r="A22" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="B22" s="8" t="s">
+      <c r="B22" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="C22" s="8" t="s">
+      <c r="C22" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="D22" s="8" t="s">
+      <c r="D22" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="E22" s="8"/>
-      <c r="F22" s="8"/>
+      <c r="E22" s="10"/>
+      <c r="F22" s="10"/>
     </row>
     <row r="23" spans="1:6">
-      <c r="A23" s="7" t="s">
+      <c r="A23" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="B23" s="7" t="s">
+      <c r="B23" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="C23" s="7">
+      <c r="C23" s="8">
         <v>50</v>
       </c>
-      <c r="D23" s="7" t="s">
+      <c r="D23" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="E23" s="7"/>
-      <c r="F23" s="7"/>
+      <c r="E23" s="8"/>
+      <c r="F23" s="8"/>
     </row>
     <row r="24" spans="1:6">
-      <c r="A24" s="7" t="s">
+      <c r="A24" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="B24" s="7" t="s">
+      <c r="B24" s="8" t="s">
         <v>103</v>
       </c>
-      <c r="C24" s="7">
+      <c r="C24" s="8">
         <v>100</v>
       </c>
-      <c r="D24" s="7" t="s">
+      <c r="D24" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="E24" s="7"/>
-      <c r="F24" s="7"/>
+      <c r="E24" s="8"/>
+      <c r="F24" s="8"/>
     </row>
     <row r="25" spans="1:6">
-      <c r="A25" s="7" t="s">
+      <c r="A25" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="B25" s="7" t="s">
+      <c r="B25" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="C25" s="7">
+      <c r="C25" s="8">
         <v>140</v>
       </c>
-      <c r="D25" s="7" t="s">
+      <c r="D25" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="E25" s="7"/>
-      <c r="F25" s="7"/>
+      <c r="E25" s="8"/>
+      <c r="F25" s="8"/>
     </row>
     <row r="26" spans="1:6">
-      <c r="A26" s="7" t="s">
+      <c r="A26" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="B26" s="7" t="s">
+      <c r="B26" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="C26" s="7">
+      <c r="C26" s="8">
         <v>150</v>
       </c>
-      <c r="D26" s="7" t="s">
+      <c r="D26" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="E26" s="7"/>
-      <c r="F26" s="7"/>
+      <c r="E26" s="8"/>
+      <c r="F26" s="8"/>
     </row>
     <row r="27" spans="1:6">
-      <c r="A27" s="7" t="s">
+      <c r="A27" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="B27" s="7" t="s">
+      <c r="B27" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="C27" s="7">
+      <c r="C27" s="8">
         <v>200</v>
       </c>
-      <c r="D27" s="7" t="s">
+      <c r="D27" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="E27" s="7"/>
-      <c r="F27" s="7"/>
+      <c r="E27" s="8"/>
+      <c r="F27" s="8"/>
     </row>
     <row r="28" spans="1:6">
-      <c r="A28" s="7" t="s">
+      <c r="A28" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="B28" s="7" t="s">
+      <c r="B28" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="C28" s="7">
+      <c r="C28" s="8">
         <v>201</v>
       </c>
-      <c r="D28" s="7" t="s">
+      <c r="D28" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="E28" s="7"/>
-      <c r="F28" s="7"/>
+      <c r="E28" s="8"/>
+      <c r="F28" s="8"/>
     </row>
     <row r="29" spans="1:6">
-      <c r="A29" s="7" t="s">
+      <c r="A29" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="B29" s="7" t="s">
+      <c r="B29" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="C29" s="7">
+      <c r="C29" s="8">
         <v>-10</v>
       </c>
-      <c r="D29" s="7" t="s">
+      <c r="D29" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="E29" s="7"/>
-      <c r="F29" s="7"/>
+      <c r="E29" s="8"/>
+      <c r="F29" s="8"/>
     </row>
     <row r="30" spans="1:6">
-      <c r="A30" s="7" t="s">
+      <c r="A30" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="B30" s="7" t="s">
+      <c r="B30" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="C30" s="7" t="s">
+      <c r="C30" s="8" t="s">
         <v>114</v>
       </c>
-      <c r="D30" s="7" t="s">
+      <c r="D30" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="E30" s="7"/>
-      <c r="F30" s="7"/>
+      <c r="E30" s="8"/>
+      <c r="F30" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3132,7 +3087,7 @@
       <c r="B2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D2" s="3" t="s">
@@ -3155,10 +3110,10 @@
       <c r="C4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="4">
         <v>46028</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="2" t="s">
         <v>11</v>
       </c>
       <c r="F4" s="3" t="s">
@@ -3166,90 +3121,90 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="5" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="7" ht="29" spans="1:5">
-      <c r="A7" s="7">
+      <c r="A7" s="8">
         <v>1</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="8" t="s">
         <v>116</v>
       </c>
-      <c r="D7" s="7">
+      <c r="D7" s="8">
         <v>1</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="8" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="8" ht="29" spans="1:5">
-      <c r="A8" s="7">
+      <c r="A8" s="8">
         <v>2</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="8" t="s">
         <v>118</v>
       </c>
-      <c r="D8" s="7">
+      <c r="D8" s="8">
         <v>2</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="8" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="7">
+      <c r="A9" s="8">
         <v>3</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="8" t="s">
         <v>120</v>
       </c>
-      <c r="D9" s="7">
+      <c r="D9" s="8">
         <v>3</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="8" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="10" spans="4:5">
-      <c r="D10" s="7">
+      <c r="D10" s="8">
         <v>4</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="8" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="11" spans="4:5">
-      <c r="D11" s="7">
+      <c r="D11" s="8">
         <v>5</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="E11" s="8" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="12" spans="4:5">
-      <c r="D12" s="7">
+      <c r="D12" s="8">
         <v>6</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="E12" s="8" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="13" spans="4:5">
-      <c r="D13" s="7">
+      <c r="D13" s="8">
         <v>7</v>
       </c>
-      <c r="E13" s="7" t="s">
+      <c r="E13" s="8" t="s">
         <v>125</v>
       </c>
     </row>
@@ -3309,132 +3264,132 @@
       </c>
     </row>
     <row r="24" spans="1:6">
-      <c r="A24" s="8" t="s">
+      <c r="A24" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="B24" s="8" t="s">
+      <c r="B24" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="C24" s="8" t="s">
+      <c r="C24" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="D24" s="8" t="s">
+      <c r="D24" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="E24" s="8"/>
-      <c r="F24" s="8"/>
+      <c r="E24" s="10"/>
+      <c r="F24" s="10"/>
     </row>
     <row r="25" spans="1:6">
-      <c r="A25" s="7" t="s">
+      <c r="A25" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="B25" s="7" t="s">
+      <c r="B25" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="C25" s="7">
+      <c r="C25" s="8">
         <v>20</v>
       </c>
-      <c r="D25" s="7" t="s">
+      <c r="D25" s="8" t="s">
         <v>132</v>
       </c>
-      <c r="E25" s="7"/>
-      <c r="F25" s="7"/>
+      <c r="E25" s="8"/>
+      <c r="F25" s="8"/>
     </row>
     <row r="26" spans="1:6">
-      <c r="A26" s="7" t="s">
+      <c r="A26" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="B26" s="7" t="s">
+      <c r="B26" s="8" t="s">
         <v>133</v>
       </c>
-      <c r="C26" s="7">
+      <c r="C26" s="8">
         <v>25</v>
       </c>
-      <c r="D26" s="7" t="s">
+      <c r="D26" s="8" t="s">
         <v>132</v>
       </c>
-      <c r="E26" s="7"/>
-      <c r="F26" s="7"/>
+      <c r="E26" s="8"/>
+      <c r="F26" s="8"/>
     </row>
     <row r="27" spans="1:6">
-      <c r="A27" s="7" t="s">
+      <c r="A27" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="B27" s="7" t="s">
+      <c r="B27" s="8" t="s">
         <v>134</v>
       </c>
-      <c r="C27" s="7">
+      <c r="C27" s="8">
         <v>26</v>
       </c>
-      <c r="D27" s="7" t="s">
+      <c r="D27" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="E27" s="7"/>
-      <c r="F27" s="7"/>
+      <c r="E27" s="8"/>
+      <c r="F27" s="8"/>
     </row>
     <row r="28" spans="1:6">
-      <c r="A28" s="7" t="s">
+      <c r="A28" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="B28" s="7" t="s">
+      <c r="B28" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="C28" s="7">
+      <c r="C28" s="8">
         <v>30</v>
       </c>
-      <c r="D28" s="7" t="s">
+      <c r="D28" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="E28" s="7"/>
-      <c r="F28" s="7"/>
+      <c r="E28" s="8"/>
+      <c r="F28" s="8"/>
     </row>
     <row r="29" spans="1:6">
-      <c r="A29" s="7" t="s">
+      <c r="A29" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="B29" s="7" t="s">
+      <c r="B29" s="8" t="s">
         <v>137</v>
       </c>
-      <c r="C29" s="7">
+      <c r="C29" s="8">
         <v>19</v>
       </c>
-      <c r="D29" s="7" t="s">
+      <c r="D29" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="E29" s="7"/>
-      <c r="F29" s="7"/>
+      <c r="E29" s="8"/>
+      <c r="F29" s="8"/>
     </row>
     <row r="30" spans="1:6">
-      <c r="A30" s="7" t="s">
+      <c r="A30" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="B30" s="7" t="s">
+      <c r="B30" s="8" t="s">
         <v>138</v>
       </c>
-      <c r="C30" s="7">
+      <c r="C30" s="8">
         <v>31</v>
       </c>
-      <c r="D30" s="7" t="s">
+      <c r="D30" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="E30" s="7"/>
-      <c r="F30" s="7"/>
+      <c r="E30" s="8"/>
+      <c r="F30" s="8"/>
     </row>
     <row r="31" spans="1:6">
-      <c r="A31" s="7" t="s">
+      <c r="A31" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="B31" s="7" t="s">
+      <c r="B31" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="C31" s="7" t="s">
+      <c r="C31" s="8" t="s">
         <v>114</v>
       </c>
-      <c r="D31" s="7" t="s">
+      <c r="D31" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="E31" s="7"/>
-      <c r="F31" s="7"/>
+      <c r="E31" s="8"/>
+      <c r="F31" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3478,7 +3433,7 @@
       <c r="B2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D2" s="3" t="s">
@@ -3501,10 +3456,10 @@
       <c r="C4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="4">
         <v>46028</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="2" t="s">
         <v>11</v>
       </c>
       <c r="F4" s="3" t="s">
@@ -3512,92 +3467,92 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="5" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="7" ht="29" spans="1:5">
-      <c r="A7" s="7">
+      <c r="A7" s="8">
         <v>1</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="D7" s="7">
+      <c r="D7" s="8">
         <v>1</v>
       </c>
-      <c r="E7" s="7">
+      <c r="E7" s="8">
         <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="7">
+      <c r="A8" s="8">
         <v>2</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="D8" s="7">
+      <c r="D8" s="8">
         <v>2</v>
       </c>
-      <c r="E8" s="7">
+      <c r="E8" s="8">
         <v>10</v>
       </c>
     </row>
     <row r="9" spans="4:5">
-      <c r="D9" s="7">
+      <c r="D9" s="8">
         <v>3</v>
       </c>
-      <c r="E9" s="7">
+      <c r="E9" s="8">
         <v>15</v>
       </c>
     </row>
     <row r="10" spans="4:5">
-      <c r="D10" s="7">
+      <c r="D10" s="8">
         <v>4</v>
       </c>
-      <c r="E10" s="7">
+      <c r="E10" s="8">
         <v>20</v>
       </c>
     </row>
     <row r="11" spans="4:5">
-      <c r="D11" s="7">
+      <c r="D11" s="8">
         <v>5</v>
       </c>
-      <c r="E11" s="7">
+      <c r="E11" s="8">
         <v>30</v>
       </c>
     </row>
     <row r="12" spans="4:5">
-      <c r="D12" s="7">
+      <c r="D12" s="8">
         <v>6</v>
       </c>
-      <c r="E12" s="7">
+      <c r="E12" s="8">
         <v>31</v>
       </c>
     </row>
     <row r="13" spans="4:5">
-      <c r="D13" s="7">
+      <c r="D13" s="8">
         <v>7</v>
       </c>
-      <c r="E13" s="7">
+      <c r="E13" s="8">
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="4:5">
-      <c r="D14" s="7">
+      <c r="D14" s="8">
         <v>8</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="E14" s="8" t="s">
         <v>114</v>
       </c>
     </row>
@@ -3644,7 +3599,7 @@
       <c r="B22" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C22" s="9" t="s">
+      <c r="C22" s="11" t="s">
         <v>146</v>
       </c>
     </row>
@@ -3665,148 +3620,148 @@
       </c>
     </row>
     <row r="26" spans="1:6">
-      <c r="A26" s="8" t="s">
+      <c r="A26" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="B26" s="8" t="s">
+      <c r="B26" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="C26" s="8" t="s">
+      <c r="C26" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="D26" s="8" t="s">
+      <c r="D26" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="E26" s="8"/>
-      <c r="F26" s="8"/>
+      <c r="E26" s="10"/>
+      <c r="F26" s="10"/>
     </row>
     <row r="27" spans="1:6">
-      <c r="A27" s="7" t="s">
+      <c r="A27" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="B27" s="7" t="s">
+      <c r="B27" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="C27" s="7">
+      <c r="C27" s="8">
         <v>5</v>
       </c>
-      <c r="D27" s="7" t="s">
+      <c r="D27" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="E27" s="7"/>
-      <c r="F27" s="7"/>
+      <c r="E27" s="8"/>
+      <c r="F27" s="8"/>
     </row>
     <row r="28" spans="1:6">
-      <c r="A28" s="7" t="s">
+      <c r="A28" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="B28" s="7" t="s">
+      <c r="B28" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="C28" s="7">
+      <c r="C28" s="8">
         <v>10</v>
       </c>
-      <c r="D28" s="7" t="s">
+      <c r="D28" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="E28" s="7"/>
-      <c r="F28" s="7"/>
+      <c r="E28" s="8"/>
+      <c r="F28" s="8"/>
     </row>
     <row r="29" spans="1:6">
-      <c r="A29" s="7" t="s">
+      <c r="A29" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="B29" s="7" t="s">
+      <c r="B29" s="8" t="s">
         <v>149</v>
       </c>
-      <c r="C29" s="7">
+      <c r="C29" s="8">
         <v>15</v>
       </c>
-      <c r="D29" s="7" t="s">
+      <c r="D29" s="8" t="s">
         <v>150</v>
       </c>
-      <c r="E29" s="7"/>
-      <c r="F29" s="7"/>
+      <c r="E29" s="8"/>
+      <c r="F29" s="8"/>
     </row>
     <row r="30" spans="1:6">
-      <c r="A30" s="7" t="s">
+      <c r="A30" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="B30" s="7" t="s">
+      <c r="B30" s="8" t="s">
         <v>151</v>
       </c>
-      <c r="C30" s="7">
+      <c r="C30" s="8">
         <v>20</v>
       </c>
-      <c r="D30" s="7" t="s">
+      <c r="D30" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="E30" s="7"/>
-      <c r="F30" s="7"/>
+      <c r="E30" s="8"/>
+      <c r="F30" s="8"/>
     </row>
     <row r="31" spans="1:6">
-      <c r="A31" s="7" t="s">
+      <c r="A31" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="B31" s="7" t="s">
+      <c r="B31" s="8" t="s">
         <v>151</v>
       </c>
-      <c r="C31" s="7">
+      <c r="C31" s="8">
         <v>30</v>
       </c>
-      <c r="D31" s="7" t="s">
+      <c r="D31" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="E31" s="7"/>
-      <c r="F31" s="7"/>
+      <c r="E31" s="8"/>
+      <c r="F31" s="8"/>
     </row>
     <row r="32" spans="1:6">
-      <c r="A32" s="7" t="s">
+      <c r="A32" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="B32" s="7" t="s">
+      <c r="B32" s="8" t="s">
         <v>152</v>
       </c>
-      <c r="C32" s="7">
+      <c r="C32" s="8">
         <v>31</v>
       </c>
-      <c r="D32" s="7" t="s">
+      <c r="D32" s="8" t="s">
         <v>150</v>
       </c>
-      <c r="E32" s="7"/>
-      <c r="F32" s="7"/>
+      <c r="E32" s="8"/>
+      <c r="F32" s="8"/>
     </row>
     <row r="33" spans="1:6">
-      <c r="A33" s="7" t="s">
+      <c r="A33" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="B33" s="7" t="s">
+      <c r="B33" s="8" t="s">
         <v>153</v>
       </c>
-      <c r="C33" s="7">
+      <c r="C33" s="8">
         <v>0</v>
       </c>
-      <c r="D33" s="7" t="s">
+      <c r="D33" s="8" t="s">
         <v>150</v>
       </c>
-      <c r="E33" s="7"/>
-      <c r="F33" s="7"/>
+      <c r="E33" s="8"/>
+      <c r="F33" s="8"/>
     </row>
     <row r="34" spans="1:6">
-      <c r="A34" s="7" t="s">
+      <c r="A34" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="B34" s="7" t="s">
+      <c r="B34" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="C34" s="7" t="s">
+      <c r="C34" s="8" t="s">
         <v>114</v>
       </c>
-      <c r="D34" s="7" t="s">
+      <c r="D34" s="8" t="s">
         <v>150</v>
       </c>
-      <c r="E34" s="7"/>
-      <c r="F34" s="7"/>
+      <c r="E34" s="8"/>
+      <c r="F34" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3850,7 +3805,7 @@
       <c r="B2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D2" s="3" t="s">
@@ -3873,10 +3828,10 @@
       <c r="C4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="4">
         <v>46028</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="2" t="s">
         <v>11</v>
       </c>
       <c r="F4" s="3" t="s">
@@ -3884,125 +3839,105 @@
       </c>
     </row>
     <row r="6" ht="29" spans="1:7">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="5" t="s">
         <v>14</v>
       </c>
       <c r="D6" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="6" t="s">
         <v>156</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="F6" s="7"/>
+      <c r="G6" s="7"/>
+    </row>
+    <row r="7" ht="29" spans="1:7">
+      <c r="A7" s="8">
+        <v>1</v>
+      </c>
+      <c r="B7" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="D7" s="9">
+        <v>1</v>
+      </c>
+      <c r="E7" s="9" t="s">
         <v>158</v>
       </c>
-      <c r="G6" s="6" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="7" ht="29" spans="1:7">
-      <c r="A7" s="7">
-        <v>1</v>
-      </c>
-      <c r="B7" s="7" t="s">
+      <c r="F7" s="8"/>
+      <c r="G7" s="8"/>
+    </row>
+    <row r="8" ht="29" spans="1:7">
+      <c r="A8" s="8">
+        <v>2</v>
+      </c>
+      <c r="B8" s="8" t="s">
         <v>159</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D8" s="9">
+        <v>2</v>
+      </c>
+      <c r="E8" s="9" t="s">
         <v>160</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="F8" s="8"/>
+      <c r="G8" s="8"/>
+    </row>
+    <row r="9" ht="29" spans="1:7">
+      <c r="A9" s="8">
+        <v>3</v>
+      </c>
+      <c r="B9" s="8" t="s">
         <v>161</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="D9" s="9">
+        <v>3</v>
+      </c>
+      <c r="E9" s="9" t="s">
         <v>162</v>
       </c>
-      <c r="G7" s="7" t="s">
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
+    </row>
+    <row r="10" spans="4:7">
+      <c r="D10" s="9">
+        <v>4</v>
+      </c>
+      <c r="E10" s="9" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="8" ht="29" spans="1:7">
-      <c r="A8" s="7">
-        <v>2</v>
-      </c>
-      <c r="B8" s="7" t="s">
+      <c r="F10" s="8"/>
+      <c r="G10" s="8"/>
+    </row>
+    <row r="11" spans="4:7">
+      <c r="D11" s="9">
+        <v>5</v>
+      </c>
+      <c r="E11" s="9" t="s">
         <v>164</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="F11" s="8"/>
+      <c r="G11" s="8"/>
+    </row>
+    <row r="12" ht="29" spans="4:7">
+      <c r="D12" s="9">
+        <v>6</v>
+      </c>
+      <c r="E12" s="9" t="s">
         <v>165</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="F12" s="8"/>
+      <c r="G12" s="8"/>
+    </row>
+    <row r="13" ht="29" spans="4:5">
+      <c r="D13" s="9">
+        <v>7</v>
+      </c>
+      <c r="E13" s="9" t="s">
         <v>166</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>167</v>
-      </c>
-      <c r="G8" s="7" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="9" ht="29" spans="1:7">
-      <c r="A9" s="7">
-        <v>3</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>170</v>
-      </c>
-      <c r="E9" s="7" t="s">
-        <v>161</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>171</v>
-      </c>
-      <c r="G9" s="7" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="10" ht="29" spans="4:7">
-      <c r="D10" s="7" t="s">
-        <v>173</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>174</v>
-      </c>
-      <c r="F10" s="7" t="s">
-        <v>175</v>
-      </c>
-      <c r="G10" s="7" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="11" spans="4:7">
-      <c r="D11" s="7" t="s">
-        <v>177</v>
-      </c>
-      <c r="E11" s="7" t="s">
-        <v>166</v>
-      </c>
-      <c r="F11" s="7" t="s">
-        <v>178</v>
-      </c>
-      <c r="G11" s="7" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="12" spans="4:7">
-      <c r="D12" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="E12" s="7" t="s">
-        <v>166</v>
-      </c>
-      <c r="F12" s="7" t="s">
-        <v>181</v>
-      </c>
-      <c r="G12" s="7" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="14" spans="1:1">
@@ -4020,7 +3955,7 @@
         <v>28</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>182</v>
+        <v>167</v>
       </c>
     </row>
     <row r="17" spans="2:3">
@@ -4028,7 +3963,7 @@
         <v>30</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>183</v>
+        <v>168</v>
       </c>
     </row>
     <row r="18" spans="2:3">
@@ -4036,7 +3971,7 @@
         <v>32</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>184</v>
+        <v>169</v>
       </c>
     </row>
     <row r="19" spans="2:3">
@@ -4044,7 +3979,7 @@
         <v>99</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>185</v>
+        <v>170</v>
       </c>
     </row>
     <row r="20" spans="2:2">
@@ -4057,7 +3992,7 @@
         <v>28</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>186</v>
+        <v>171</v>
       </c>
     </row>
     <row r="22" spans="2:3">
@@ -4065,7 +4000,7 @@
         <v>30</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>187</v>
+        <v>172</v>
       </c>
     </row>
     <row r="23" spans="2:3">
@@ -4073,7 +4008,7 @@
         <v>32</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>188</v>
+        <v>173</v>
       </c>
     </row>
     <row r="24" spans="2:3">
@@ -4081,120 +4016,120 @@
         <v>99</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>188</v>
+        <v>173</v>
       </c>
     </row>
     <row r="26" spans="1:6">
-      <c r="A26" s="8" t="s">
+      <c r="A26" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="B26" s="8" t="s">
+      <c r="B26" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="C26" s="8" t="s">
-        <v>189</v>
-      </c>
-      <c r="D26" s="8" t="s">
+      <c r="C26" s="10" t="s">
+        <v>174</v>
+      </c>
+      <c r="D26" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="E26" s="8"/>
-      <c r="F26" s="8"/>
+      <c r="E26" s="10"/>
+      <c r="F26" s="10"/>
     </row>
     <row r="27" spans="1:6">
-      <c r="A27" s="7" t="s">
+      <c r="A27" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="B27" s="7" t="s">
-        <v>190</v>
-      </c>
-      <c r="C27" s="7" t="s">
-        <v>191</v>
-      </c>
-      <c r="D27" s="7" t="s">
-        <v>192</v>
-      </c>
-      <c r="E27" s="7"/>
-      <c r="F27" s="7"/>
+      <c r="B27" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="D27" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="E27" s="8"/>
+      <c r="F27" s="8"/>
     </row>
     <row r="28" spans="1:6">
-      <c r="A28" s="7" t="s">
+      <c r="A28" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="B28" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="C28" s="7" t="s">
-        <v>194</v>
-      </c>
-      <c r="D28" s="7" t="s">
-        <v>168</v>
-      </c>
-      <c r="E28" s="7"/>
-      <c r="F28" s="7"/>
+      <c r="B28" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="C28" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="D28" s="8" t="s">
+        <v>180</v>
+      </c>
+      <c r="E28" s="8"/>
+      <c r="F28" s="8"/>
     </row>
     <row r="29" spans="1:6">
-      <c r="A29" s="7" t="s">
+      <c r="A29" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="B29" s="7" t="s">
-        <v>195</v>
-      </c>
-      <c r="C29" s="7" t="s">
-        <v>196</v>
-      </c>
-      <c r="D29" s="7" t="s">
+      <c r="B29" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="C29" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="D29" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="E29" s="7"/>
-      <c r="F29" s="7"/>
+      <c r="E29" s="8"/>
+      <c r="F29" s="8"/>
     </row>
     <row r="30" spans="1:6">
-      <c r="A30" s="7" t="s">
+      <c r="A30" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="B30" s="7" t="s">
-        <v>197</v>
-      </c>
-      <c r="C30" s="7" t="s">
-        <v>174</v>
-      </c>
-      <c r="D30" s="7" t="s">
+      <c r="B30" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="C30" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="D30" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="E30" s="7"/>
-      <c r="F30" s="7"/>
+      <c r="E30" s="8"/>
+      <c r="F30" s="8"/>
     </row>
     <row r="31" spans="1:6">
-      <c r="A31" s="7" t="s">
+      <c r="A31" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="B31" s="7" t="s">
-        <v>198</v>
-      </c>
-      <c r="C31" s="7">
+      <c r="B31" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="C31" s="8">
         <v>11</v>
       </c>
-      <c r="D31" s="7" t="s">
+      <c r="D31" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="E31" s="7"/>
-      <c r="F31" s="7"/>
+      <c r="E31" s="8"/>
+      <c r="F31" s="8"/>
     </row>
     <row r="32" spans="1:6">
-      <c r="A32" s="7" t="s">
+      <c r="A32" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="B32" s="7" t="s">
-        <v>199</v>
-      </c>
-      <c r="C32" s="7">
+      <c r="B32" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="C32" s="8">
         <v>-1</v>
       </c>
-      <c r="D32" s="7" t="s">
+      <c r="D32" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="E32" s="7"/>
-      <c r="F32" s="7"/>
+      <c r="E32" s="8"/>
+      <c r="F32" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>